<commit_message>
feat: simplify Vietnam replenishment settings and CLI execution
</commit_message>
<xml_diff>
--- a/python/lxeskill_cli/services/vietnam_replenishment/resources/skeleton.xlsx
+++ b/python/lxeskill_cli/services/vietnam_replenishment/resources/skeleton.xlsx
@@ -999,7 +999,7 @@
         <v/>
       </c>
       <c r="S2" s="28">
-        <f>K2*0.1/(30+AV2)+L2*0.3/(15+AW2)+M2*0.6/(7+AX2)</f>
+        <f>K2*数据更改!$E$2/(30+AV2)+L2*数据更改!$F$2/(15+AW2)+M2*数据更改!$G$2/(7+AX2)</f>
         <v/>
       </c>
       <c r="T2" s="29">
@@ -1110,7 +1110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1183,7 +1183,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:M2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1196,7 +1195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1284,7 +1283,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:P2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1297,7 +1295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1321,6 +1319,21 @@
           <t>汇率</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>30天销量权重</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>15天销量权重</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>7天销量权重</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="43" t="n">
@@ -1334,6 +1347,15 @@
       </c>
       <c r="D2" s="43" t="n">
         <v>3900</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -1347,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1412,7 +1434,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
   </sheetData>
   <autoFilter ref="A1:K2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: configure Vietnam sales weights and day adjustments
</commit_message>
<xml_diff>
--- a/python/lxeskill_cli/services/vietnam_replenishment/resources/skeleton.xlsx
+++ b/python/lxeskill_cli/services/vietnam_replenishment/resources/skeleton.xlsx
@@ -999,7 +999,7 @@
         <v/>
       </c>
       <c r="S2" s="28">
-        <f>K2*0.1/(30+AV2)+L2*0.3/(15+AW2)+M2*0.6/(7+AX2)</f>
+        <f>K2*数据更改!$E$2/(30+AV2)+L2*数据更改!$F$2/(15+AW2)+M2*数据更改!$G$2/(7+AX2)</f>
         <v/>
       </c>
       <c r="T2" s="29">
@@ -1297,7 +1297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
@@ -1321,6 +1321,21 @@
           <t>汇率</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>30天销量权重</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>15天销量权重</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>7天销量权重</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="43" t="n">
@@ -1334,6 +1349,15 @@
       </c>
       <c r="D2" s="43" t="n">
         <v>3900</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>